<commit_message>
Apply the supplied Smart Pursuit logo to all 21 audits and the workbook
- assets/smart-pursuit-logo.png (the circular SMART PURSUIT lockup, uploaded by the
  client) is now embedded on the cover and on every body page of all 21 audits,
  top-left, and on the workbook README sheet.
- assets/smart-pursuit-logo.mode.txt = lockup: the logo already carries the wordmark,
  so the report no longer prints 'SMART PURSUIT' beside it (cover and page headers).
- Cover mark sized 16 mm and left-aligned with the rest of the cover.
- Verified: image embedded on every page of all 21 PDFs (116 pages), footer/logo/header
  checks pass, and the text of every audit is byte-identical to the previous build once
  the old drawn mark is discounted - no content changed.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/niches/food-bengaluru/Food-Bangalore-ALL-IN-ONE.xlsx
+++ b/niches/food-bengaluru/Food-Bangalore-ALL-IN-ONE.xlsx
@@ -263,6 +263,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="1428750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -775,6 +805,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add flat Emails sheet from leads/*.json
</commit_message>
<xml_diff>
--- a/niches/food-bengaluru/Food-Bangalore-ALL-IN-ONE.xlsx
+++ b/niches/food-bengaluru/Food-Bangalore-ALL-IN-ONE.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leaks &amp; Roadmap" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="You vs Competitor" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected ROI" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Basis (sources)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills Used" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings (severity+evidence)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunity Score" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage (measured vs not)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verify These (links)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cannot be verified" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Leads" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Emails" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Leaks &amp; Roadmap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="You vs Competitor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Expected ROI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Audit Basis (sources)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Skills Used" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Findings (severity+evidence)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Opportunity Score" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Coverage (measured vs not)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Evidence Register" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Verify These (links)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Cannot be verified" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Emails (one sheet)" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$O$22</definedName>
@@ -263,36 +264,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>3</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="1428750"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,7 +579,6 @@
       <c r="B2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
@@ -672,7 +642,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
@@ -744,7 +713,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -805,7 +773,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -16118,6 +16085,1316 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Brand name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Body 1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Body 2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Body 3</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Body 4</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Attachment Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>support@akshayakalpa.org</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: ~400 live ads - and a California placeholder address on the landing page
+Day 3: The problem with 400 creatives
+Day 7: You are turning away B2B demand
+Day 14: Closing the file on Akshayakalpa</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for food brands from Bengaluru. Your footprint is the biggest I found in this category: ~400 live Google creatives under Akshayakalpa Farms and Foods Pvt Ltd. The product story behind it is world-class - 4C farm chilling, 24-36 hours to doorstep vs the 72-96 hour industry norm, APEDA certified.
+One thing you can check in 30 seconds: the Contact Us page at akshayakalpa.org/contact-us currently contains template placeholder text - '0123.456.789 - 2 Queen Street, California, USA'. Your paid traffic lands on that page. It is a small fix and a direct trust cost while it is live.
+Attached is the 7-page Paid Media and Measurement Audit, including what I would do with ~400 creatives to make them learn faster than they spend. Worth 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220
+P.S. I am writing to your published support address because the site does not list a marketing or partner contact - that is itself one of the findings.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following up on the audit. At ~400 creatives, the risk is not lack of creative - it is that nobody can name the top 10 performers, so the other 390 keep paying for lessons you already learned.
+The fix is boring and effective: instrument everything, rank by CPA, cut the bottom third, and rebuild around three repeatable formats from one shoot day per week. Same budget, much sharper inventory.
+I can show you the ranking framework we use - it takes about 20 minutes to walk through.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+One more finding. Organic dairy has natural B2B lines - cafes, cloud kitchens, hotels, corporate pantry, gifting - and your site publishes only a support number. A distributor or a 200-box gifting enquiry has nowhere to land.
+A simple enquiry page plus a small always-on campaign would open a revenue line you are currently refusing, at a fraction of the cost of new consumer acquisition.
+Happy to map the flow (form, follow-up, pricing-on-request).
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note from me. The audit's three fixes: (1) clean the funnel and rebuild the top landing pages around your 24-36 hour freshness proof, (2) rank and prune the 400-creative inventory into a weekly system, (3) open B2B and gifting enquiry paths.
+The audit is yours to keep. If you would like help, we would start with the creative ranking - it usually pays for itself in the first fortnight.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>akshayakalpa-organic-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>care@anandsweets.net</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your ads are sending buyers to Swiggy - the Anand Sweets audit
+Day 3: Corporate gifting is your highest-value leak
+Day 7: Own the festival calendar in Bengaluru
+Day 14: Closing the file on Anand Sweets</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I run paid-media audits for Bengaluru food brands. I checked your live footprint: 58 Google creatives under Anand Sweets &amp; Savouries LLP, and Google shows you as a Verified advertiser - a real asset in mithai, where trust decides the order.
+The problem: your own top banner tells every paid visitor that Bangalore delivery takes up to 3 days and sends same-day buyers to Swiggy, Zomato or Ownly. That is the exact moment - festive, urgent, gift-driven - where mithai margins live, and it is being handed to an aggregator.
+Attached is the 7-page Paid Media and Measurement Audit. Open to a 15-minute call?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding from the audit: corporate and wedding gifting are your highest order values, and they are reached by browsing - not by paid campaigns.
+A dedicated gifting campaign (search for 'corporate Diwali gifts Bangalore', Meta lookalikes, LinkedIn for HR/admin) landing on the corporate page with GST invoice, custom branding and care@anandsweets.net in the first screen would turn this into a pipeline instead of a page.
+One 500-box order pays for the campaign many times over. I can share the full structure.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+With 15+ stores and 58 live creatives, you are a paid-media leader in this category - but festival demand is still fought on broad audiences.
+The playbook: a 12-month occasion calendar (Diwali, Ugadi, Sankranti, wedding season) with pre-built creatives, geo-radius audiences around each store, and cart-abandonment retargeting. One store radius = one local ad set, measured per store.
+Happy to walk through the calendar we would build for you.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit stands on three fixes - (1) keep same-day demand on your own domain with pickup/express instead of routing to Swiggy, (2) run corporate gifting as a campaign, (3) build the festival calendar with per-store geo audiences and cart retargeting.
+The document is yours regardless. If you would like us to implement the gifting campaign first, we can start next week.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>anand-sweets-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Barbeque Nation</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>feedback@barbequenation.com</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 15 creatives on your domain that are not yours (and a code mismatch)
+Day 3: Five URLs your printed material probably still points at
+Day 7: Your offers are not visible in your own reporting
+Day 14: Closing the file on Barbeque Nation</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. Two findings from this week's live data:
+1. 34 creatives point at barbequenation.com, but only 19 sit in the United Foodbrands account — the other 15 come from other accounts. Usually franchise or partner buying, but worth knowing.
+2. Your running takeaway ad says 'Use code SAVE35' in the copy and 'Use Code SAVE5' in the image inside the same ad.
+The attached audit documents both, with the URLs to check them yourself.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second note. /menu, /locations, /book-a-table, /order-online and /terms all return 404 today. Your ad destinations are fine — /ubq-delivery and /deals/unlockspecialdeals both work — but every QR code, menu card and old blog link that uses the conventional URLs dead-ends.
+A set of redirects fixes it in an afternoon and costs nothing.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, about measurement rather than creative. You have a tag manager, Meta's script and Razorpay in place — a sound stack. What I cannot see from outside is any event tied to the offer codes (SAVE35, or the pay-day offer expiring 11 October).
+Without that, an offer can only be judged by counting orders, which cannot separate the offer's effect from the campaign's. One dataLayer push per code settles it permanently.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note. The audit's three fixes are: align the code in the takeaway ad, redirect the five dead paths, and instrument offer-code redemption.
+We work with F&amp;B brands across Bengaluru. If a short call on any of the three is useful, I am happy to make time — and if not, the audit stands on its own.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>barbeque-nation-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Milky Mist</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>customercare@milkymist.com</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 3 live Google ads for an IPO-bound dairy major
+Day 3: The dairy subscription you are not selling
+Day 7: Two websites, two journeys
+Day 14: Closing the file on Milky Mist</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I run paid-media audits for food brands from Bengaluru. I checked your live presence this week: Milky Mist Dairy Food Limited shows 3 live Google creatives - while the corporate site carries a full IPO section, SEBI Reg 46 disclosures and investor pages.
+That gap matters now: paneer, curd, ghee and cheese searches are high-intent purchase moments, and today they are being answered by Amul, Nandini and quick-commerce private labels. Before a listing, demand durability is part of the story you will be asked about.
+Attached is the 7-page Paid Media and Measurement Audit. Open to 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following the audit: dairy is the most subscription-friendly category in India - milk, curd and paneer are bought weekly. A subscribe-and-save flow on the Shopify store (bundles, free-delivery threshold, WhatsApp reminders) adds predictable revenue and a much stronger demand story for the IPO window.
+It also lowers CAC permanently: subscription customers compound instead of being re-bought every month.
+I can share the offer mechanics and retention benchmarks we use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third finding from the audit. Your brand currently lives across a Wix corporate site and a separate Shopify store. Paid traffic, brand story and purchase path are split - which quietly costs conversion on every campaign.
+The fix: pick the Shopify store as the single purchase destination, keep the corporate site for brand, investor and B2B audiences, and measure per SKU family so you know exactly what the spend is buying.
+Happy to map the handoff structure.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit's three fixes are (1) build the category search moat with product-specific landing pages, (2) launch subscribe-and-save for weekly dairy, (3) unify the paid journey onto the Shopify store and measure per SKU family.
+The audit is yours to keep. If you would like to start, the search moat is the fastest measurable win.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>milky-mist-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Millet Amma</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>eatright@milletamma.com</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 80 live ads — and one of them left in Google's archive with placeholders showing
+Day 3: Two analytics properties are counting the same visitors
+Day 7: Your best trust asset is not in your ads
+Day 14: Closing the file on Millet Amma</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands, and your account stands out: 80 live Google creatives under Urban Monk Private Limited, with video and local formats in the mix.
+One thing worth fixing fast: a local-ad creative in Google's public archive still shows the template strings '{KeyWord:Millet Amma}' and '&lt;Rating (Reviews)&gt; · &lt;Distance&gt; · Bengaluru', last shown 15 July. Anyone can open it.
+The attached audit has that URL plus every measurement behind it.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding, this one numerical. Your storefront loads two GA4 properties at once — G-WH82716CE0 and G-N659GJMWCX — alongside your Ads tag. Two properties means every session is counted twice and no report agrees with another.
+Consolidating to one is an hour of work with an infrastructure-grade payoff: one number everyone can argue with.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note. Your footer says 'Watch us on Shark Tank India'. Your paid creative says 'A sweet that feels like home, without the refined sugar' — which is genuinely good copy, but it is not the credential.
+National-TV proof in the first line of a hook is a cheap test with a clear read after two weeks. Worth trying before the festive season.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. The audit comes down to: consolidate the two GA4 properties, rebuild four missing pages (FAQ, store locator, bulk, corporate gifting), and refresh the local-ad set.
+If you would like help on the measurement side first — the fastest of the three — reply and I will send a step-by-step.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>millet-amma-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Organic Mandya</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: You have the best delivery promise in the category — and none of your ads say it
+Day 3: 69 Google creatives, and roughly two Meta results
+Day 7: Your custom dataLayer is doing nothing yet
+Day 14: Closing the file on Organic Mandya</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. Your site promises 2-hour delivery in Bengaluru, Hyderabad and Mysuru (₹49 under ₹500, free above). Your live Google creative — I captured 'organic rajmudi rice (rajamudi) — karnataka's heritage red rice' — sells the product instead.
+You own a claim most organic brands cannot make. The attached audit shows where it is missing and what to test first.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. Your Google account holds 69 creatives. On Meta, the brand term returns about two active results — one of them yours, pointing at a category collection.
+Collection-level ads against a visual grocery catalogue is exactly the right structure for a basket business. Two ads is a test that was never scaled; the attached audit describes the first three campaigns I would run.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, and it is a compliment with a gap attached. Your storefront pushes custom events called gtm-promo, gtm-creative, gtm-position and gtm-destination. Someone built a real measurement plan.
+None of it changes your reports until those events are mapped to GA4 key events and imported into Google Ads. That is configuration, not development — and it is the difference between guessing and knowing which collection earns its spend.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. Three moves: put the two-hour promise into the ad copy, map the dataLayer events into conversions, and give corporate gifting a page.
+If the corporate-gifting idea interests you, I can share the page structure we use — it is the fastest of the three to prove out.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>organic-mandya-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SMOOR</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>info@smoorchocolates.com</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 22 live Google ads — and two enquiry pages that go nowhere
+Day 3: Your Shopping titles are doing too much work
+Day 7: You are selling to companies — is the quote tracked?
+Day 14: Closing the file on SMOOR</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I went through your live footprint this week: 22 Google creatives running under Bliss Chocolates India Private Limited, including Shopping ads, plus three Meta creatives selling corporate gifting into your /pages/corporate-gifting page.
+Two things worth ten minutes: /pages/contact and /pages/bulk-enquiry both return 404 today, and your live offer excludes celebration cakes — the category most people arrive for.
+The attached Paid Media &amp; Measurement Audit has the full picture, with the URL for every claim.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second thought from the audit. One of your live Shopping titles is: 'Elsa and Anna Cake | Frozen Theme Birthday Cake | Elsa &amp; Anna Kids Designer Cake | Princess Celebration Cake by SMOOR | 1.5 Kg'.
+That title is optimised for matching, not for the person reading it on a phone. A feed pass over the five longest titles usually improves click-through before any bid change — and it costs nothing.
+Happy to send the rewritten titles as a starting point.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third thought. All three of your verified Meta creatives point at the corporate-gifting page and ask for a quote. The page works; the ads are well aimed.
+What I cannot see from outside is whether a quote request fires a tracked event. If it does not, that campaign can only ever be judged on clicks. One event on the form makes the whole quarter's gifting push measurable.
+Worth a check before the Diwali window closes.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note from me. The audit's three fixes are deliberately small: redirect two dead enquiry URLs, rewrite the five longest Shopping titles, and put one tracked event behind the corporate-gifting quote form.
+If the timing is wrong, no problem — reply 'later' and I will leave it there.
+The audit is yours either way.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>smoor-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sid's Farm</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>wecare@sidsfarm.com</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Seven 404s under a paid engine that is working
+Day 3: Two settings worth checking today
+Day 7: Your Meta copy is a template for the rest of the category
+Day 14: Closing the file on Sid's Farm</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. Your paid side is genuinely good: around 200 creatives in the account, three Meta creatives verified by ID running since April and August, and an app landing URL with proper campaign macros attached.
+Underneath it, seven standard pages return 404 today — contact, FAQ, shipping policy, store locator, bulk and corporate-gifting. For a subscription where the first order is a trust decision, those are the most expensive pages on the site.
+The attached audit lists every URL and every measurement.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Two configuration findings from the audit, both verifiable in your own dashboard.
+1. Two Google Tag Manager containers load on the same page (GTM-57TDVNH and GTM-P4DXD97J). That pattern normally produces duplicated purchase or signup events.
+2. Your store config reads meta_pixel_enable: false with an empty pixel ID — while Meta ads are running. It may be fired through GTM instead, but that is worth knowing for certain.
+Both take an hour to settle and both decide whether ROAS discussions are winnable.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, this one a compliment. 'No diet changes. No extra effort. Just your everyday milk, now with 22g protein in every pack.' is the right way to sell a subscription — a product change, not a discount.
+The same story is missing on the site: the pages that explain testing have no equivalent. If you want, I will map the three pages (testing, delivery, subscription terms) against what your Meta traffic actually asks.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. The audit comes down to three fixes: publish the four missing trust pages, settle the double container and the pixel setting, and report app and website growth as one number.
+No pressure at all — if you would rather just take the page list and run with it internally, that is a perfectly good outcome.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>sid-s-farm-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>customercare@idfreshfood.com</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: INR 681 Cr revenue, one live Google ad - here is the audit
+Day 3: The category searches you are not buying
+Day 7: Subscribe-and-save is your pre-IPO revenue line
+Day 14: Closing the file on iD Fresh</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I run paid-media audits for food brands from Bengaluru. I checked your live footprint this week: Google Ads Transparency shows one live creative for idfreshfood.com, running under Blink Digital India Pvt Ltd.
+That is remarkable for a brand at INR 681 Cr revenue with an IPO in view - and it means every 'idli batter home delivery', 'malabar parota online' or 'preservative-free batter' search is being answered by quick-commerce and smaller D2C brands, not by you.
+I have attached the 7-page Paid Media and Measurement Audit, including the subscription engine that would add recurring revenue before your IPO window. 15 minutes this week?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following up: the audit recommends a search moat across brand, category and competitor terms, with three landing paths - nearest store, quick-commerce, and subscribe-and-save.
+Batter is bought weekly by the same household, so search + retargeting here is unusually profitable: you are not buying new customers, you are capturing demand that already exists in your category.
+I can send the keyword clusters and geo-split structure we would use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+One more from the audit, and it is the one I would prioritise before an IPO: weekly batter is a subscription category, and subscribe-and-save with a 10-15% incentive and WhatsApp reminders converts existing buyers into predictable recurring revenue.
+Owned D2C recurring revenue is the most valuable line you can add to the story - and paid media is the cheapest way to build it.
+Happy to map the mechanics (offer, cadence, retention curve) for you.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note: the audit's three fixes are (1) build the search moat with three landing paths, (2) launch subscribe-and-save with WhatsApp reminders, (3) turn the preservative-free process into ad creative that defends your premium.
+The audit is yours. If you want, we can start with the search structure and show results before any creative work.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>id-fresh-food-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Adukale</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>info@adukale.com</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your ads still land on a site that sends buyers to Amazon
+Day 3: Three Shopping ads are pulled — and that is usually fixable in a day
+Day 7: Two visible defects on the live storefront
+Day 14: Closing the file on Adukale</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. Your storefront now says: 'All purchases from this site will now be completed through Amazon.' At the same time, 13 Google creatives are live for adukale.com.
+That combination has an obvious cost: paid clicks that either lose the sale or hand your customer record to Amazon. The attached audit lays out the two clean ways to resolve it.
+Everything in it is dated and sourced.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. One of your archived Shopping ads shows 'Last shown: Nov 28, 2025', with all three of its variations carrying Google's notice 'Removed for a policy violation': Sambar Powder, Chutney Powder 200g and Kayi Kodubale 180g.
+PLA removals are usually feed-level — price, availability or a landing-page mismatch — and are resolved in Merchant Center. Worth knowing, because Shopping is the visible engine in your account.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, and these are two five-minute fixes on live pages. Your pickup block still shows the Shopify template address: '123 John Doe Street, Your Town, YT 12345', next to your real pickup point at Mallathalli.
+And the email icon in your footer is coded without a mailto: prefix (verbatim: &lt;a href="info@adukale.com"&gt;), so a click cannot open a mail client. The address reads correctly, which is why nobody has noticed.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note. The audit boils down to one decision — where the paid click should end while Amazon is the checkout — plus three small fixes (placeholder address, mailto, Merchant Center feed).
+If a 20-minute call on the routing question would help, I am happy to make time. Otherwise the audit is yours to use internally.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>adukale-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Araku Coffee</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>customercare@arakuoriginals.com</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: ~200 live creatives — and every Shopping click filed as organic
+Day 3: Your cafés and your store share one advertiser account
+Day 7: On Meta, your brand name returns somebody else's business first
+Day 14: Closing the file on Araku Coffee</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food and beverage brands. Your account is the largest I looked at this week: ~200 live creatives under Araku Originals Pvt Ltd, including Shopping ads for the Moka Pot and the Chemex, plus café listings with reserve actions.
+One reporting problem sits underneath all of it: every Shopping click carries utm_campaign=sag_organic, so GA4 files your paid traffic as organic. The attached audit shows the exact URL and the fix.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. In the same account I can see a local listing for 'ARAKU Coffee' with Directions and Reserve, and Shopping ads for brewing equipment landing on product pages.
+Two different businesses, one set of conversions — which means nobody can say whether a rupee bought a café visit or a bag of beans. Separating the conversion actions takes an afternoon and makes your budget conversations evidence-based.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, and it is delicate. Searching your brand term on Meta surfaces third-party placements ahead of your own — a partner workshop carrying the name, and a separately-trading café. Neither looks hostile, but it means brand search on Meta is not currently yours.
+Worth a look at the account level together with whoever manages partner activity.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. The audit's three moves: correct the sag_organic tag in the feed, separate café and e-commerce conversions, and add redirects from the conventional URL handles.
+The first is a few minutes of work with immediate effect on every report your team reads. Happy to walk someone through it if useful.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>araku-coffee-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Brik Oven</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>theteam@brikoven.com</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your store ads are excellent — and the booking click leaves your domain
+Day 3: Nine URLs your customers type, all returning 404
+Day 7: The Palace Road breakfast ad stopped in July
+Day 14: Closing the file on Brik Oven</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. Your local ads are the best-constructed set I have seen this month: store-level creatives for Manyata Business Park and Palace Road with directions, call and reserve actions.
+One structural problem: the reservation CTA goes to widget.reservego.co — so the booking data, the no-show list and the store-level attribution belong to the widget, not to you. The attached audit explains what moving it back would give you.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. /contact-us, /menu, /book-a-table, /locations and /order-online all return 404 today (along with about-us, faq, privacy-policy and terms).
+Your paid traffic is driven by store-level intent — people looking for pizza near a specific outlet. Those are exactly the visitors most likely to book, and today the obvious URLs dead-end. Redirects are an afternoon's work.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note. Google's archive shows your Palace Road breakfast creative — 'Smoked Ham Bagel Mornings — Sourdough sandwiches, bagels &amp; toasties. Open 8AM-11AM daily' — with 'Last shown: Jul 23, 2026'.
+The creative is good; it just is not running while the stores are. A monthly five-minute review of which store ads are live keeps the set earning.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. Two moves matter most here: put a booking form on your own domain, and redirect the nine dead paths. After that, a monthly review keeps the local-ad set current.
+If a short call on the booking flow would be useful, I can bring the structure we use for restaurant groups.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>brik-oven-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>customercare@chaipoint.com</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 8,100 workplaces, 150+ Brewing Bots, no paid B2B funnel
+Day 3: The Brewing Bot deserves a demo funnel
+Day 7: 150 stores, zero store-radius campaigns
+Day 14: Closing the file on Chai Point</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I checked your live footprint: 56 Google creatives under Mountain Trail Foods, a genuinely modern site (GA4 G-EN77D2S0YH), and the numbers you publish are strong - 150+ stores, 900,000 cups a day, 8,100 workplace clients.
+Here is the leak: the B2B side - your highest-value line - has no paid funnel. No 'book a demo' path for office admins searching for tea vending, while your Brewing Bot (real tea leaves, not premix) is a genuinely superior product to every coffee-only incumbent.
+Attached: the 7-page Paid Media and Measurement Audit. Worth 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following the audit: 8,100 workplaces is proof the product sells - but it is selling through people, not paid demand.
+A simple funnel - landing page with cups/day calculator and install timeline, Google search on 'office tea vending machine', LinkedIn targeting admin/HR titles, and a two-ad retargeting sequence with case studies - turns that into inbound pipeline per city.
+Happy to share the page structure and the exact targeting we would use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third finding from the audit. With 150+ stores in 19 cities, you are competing with app-first brands that buy hyperlocal inventory around their outlets. Your top Bengaluru stores should each have a 3-5 km radius campaign with a store-specific first-order offer - measured on walk-ins, not just clicks.
+25 stores is enough to build the template, prove the lift, and then scale city by city. It also gives your FICO investors a demand-generation story, not just a product story.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note from me: the audit's three fixes are (1) build the workplace/Brewing Bot demo funnel, (2) give the top 25 stores radius campaigns with store-level measurement, (3) start habit retargeting with a WhatsApp opt-in - chai is a daily drink, and that is your cheapest repeat revenue.
+The audit is yours to keep. If you want, we can start with the B2B demo funnel this month.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>chai-point-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Cothas Coffee</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>customercare@cothas.com</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 77 live Google ads, one destination - the Cothas audit
+Day 3: Your vending line is a B2B lead engine waiting to happen
+Day 7: Free creatives: your customers' morning filter coffee
+Day 14: Closing the file on Cothas</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I inspected your live footprint this week: 77 Google creatives running under Freeflow Creative Services, including Local store ads like your HMT Road Mathikere store. Genuinely good work - most heritage brands your age run zero paid.
+The gap: a cafe owner searching 'coffee vending machine', a household buying filter coffee, and someone near a CoCo outlet all land on the same destination. Three buyers, one page.
+Attachment: the 7-page Paid Media and Measurement Audit. Worth a short call?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second thought from the audit. 'Coffee vending machine' search intent is high-value and almost nobody in Indian coffee serves it with a proper page: ROI proof (cups/day, payback period), a short enquiry form, and WhatsApp handoff.
+One vending contract can be worth hundreds of D2C orders. With 77 creatives already live, you have the traffic - it just needs a destination built for that buyer.
+I can share the page structure we use for F&amp;B B2B funnels if useful.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last idea from the audit. Filter coffee is the most photographed ritual in South India, and your account barely uses customer content. A monthly #MyCothasFilter collection - 10 best photos/videos become paid creatives - gives you fresh creative every month at zero production cost, with real social proof.
+For a brand 'since 1948', customer ritual content is the strongest credibility asset you have.
+Happy to map the full 30-day plan.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up: the audit attached on Day 1 stands on three fixes - (1) split traffic into household / B2B vending / store destinations, (2) build the vending lead engine, (3) start a UGC ritual campaign.
+No pressure if now is not the time. If you want, we can start with just the vending page and the enquiry flow this month.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>cothas-coffee-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Early Foods</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>hello@earlyfoods.com</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 30 live ads for Early Foods - the trust gap in the first 5 seconds
+Day 3: Your best creative is sitting in your customers' kitchens
+Day 7: Baby food is a 2-year subscription - is it priced like one?
+Day 14: Closing the file on Early Foods</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I checked your live footprint: 30 Google creatives under Early Foods Pvt Ltd, plus a global storefront already live - strong setup for a clean-label brand.
+One finding: in baby food, parents are not choosing between brands - they are weighing the risk of trying you against a known multinational. Your ads and landing path lead with product; they should lead with reassurance: age-appropriate, full ingredient list, what is NOT inside, and other parents' faces.
+Attached: the 7-page Paid Media and Measurement Audit. Open to 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following the audit: the highest-converting asset in baby food is another parent's face and words - and there is no visible system collecting them.
+Simple version: offer a starter bundle to 50 existing customers for a 20-second video ('what I feed my 10-month-old'). Rotate the top 12 as paid creatives every month. Real kitchens, real babies, zero production cost.
+Happy to share the brief and permission/consent flow.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third finding. A parent who starts at 6 months stays 18-36 months. That predictable LTV changes everything: stage-based bundles (6m / 9m / 12m / 18m) with auto-replenish and WhatsApp reminders turn a one-off order into a two-year relationship.
+Add a 'grow with us' upgrade path and you have a retention system no multinational shelf brand can match.
+Want me to map the bundle ladder against your SKUs?
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit's three fixes are (1) trust-first, age-matched landing pages, (2) a parent UGC engine, (3) stage-based subscription bundles with WhatsApp reminders.
+Also worth a test later: you already run a global store - the UAE, Singapore and US Indian-parent audiences are reachable at low incremental cost.
+The audit is yours. If you want to start, the UGC engine is the fastest win.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>early-foods-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Eat Better Co</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>care@eatbetterco.com</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your Shopping feed is advertising 1% off
+Day 3: Your policy pages send customers to a different domain
+Day 7: You have a Meta Lead event — inside one form
+Day 14: Closing the file on Eat Better Co</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for food brands. Running through your live Shopping ads this week, three stood out: four of them carry discount badges: [-1%] on quinoa namkeen, [-2%] on the sweet crunchy nut mix and again on a ragi bundle, and [-6%] on trail mix 100g.
+A 1% badge reads as an offer and delivers a rounding error. Either removing the badge or repricing fixes it, and both are feed-level decisions made once.
+The attached audit shows the listings and everything else I measured.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. Your contact and refund pages publish care@eatbetterco.com; your privacy and shipping pages publish connect@gottaeatbetter.com.
+A customer who reads your shipping policy and then writes to that address has been sent to a domain they have never seen. One canonical address with the other as a forwarding alias solves it in minutes.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, and it is a good sign with a caveat. Your enquiry form is configured with a Meta pixel (3182482251838473) and fires a custom Lead event on submit, then sends people to your Diwali hampers collection.
+That works — but a Lead event that fires from one form only is a single point of failure, and it means the pixel cannot see any other page. The attached audit explains the two ways to extend it.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note from me. The audit's three moves: clean the sub-10% discounts out of the feed, put one support address across the site, and test the Shark Tank line plus the ₹500 free-shipping threshold in the ad copy.
+No reply needed if the timing is wrong — the audit is yours either way.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>eat-better-co-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>talktous@licious.com</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your Bengaluru Meta ad lands on a store-locator - here is the audit
+Day 3: The cheapest fix in the Licious audit
+Day 7: Why your Google spend is thinning out
+Day 14: Closing the file on Licious</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I run paid-media audits for food brands out of Bengaluru. Over the last few days I inspected your live ad footprint - not a guess: Google Ads Transparency shows ~300 creatives under Delightful Gourmet Pvt Ltd, and I verified your Meta flight live in the Ad Library (Library ID 983369480870934, running since 15 Apr 2026).
+One finding you can act on today: that live Meta ad sends Bengaluru clicks to licious.in/store-locator. Buyers who tapped because of 'never frozen' arrive at a city picker - one full step before they see a product or price.
+I have attached the 7-page Paid Media and Measurement Audit, all doable without increasing spend. Worth 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220
+P.S. The 0-4C cold-chain story is genuinely your strongest asset. It deserves to be the hero of the landing page, not just the ad.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following up on the audit. If you only do one thing this week: take your 5 biggest-spend Bengaluru Meta ads and repoint them from the store-locator to the SKU page with city_id=1 pre-set.
+It needs no new creative, no new budget - and it removes the single most expensive step between the tap and the cart. Keep the locator as the secondary CTA.
+Happy to send the exact URL pattern and the UTM setup we use so your comparison stays clean for 14 days.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second observation from the audit: with ~300 Google creatives live - including a large Local store-ad layer - budget gets spread thinly across assets and geos. Concentrating spend on the SKU/geo clusters that match your cold-chain promise typically beats adding creatives.
+We build this exact consolidation + creative-refresh system for food brands: one shoot day a week, three formats, weekly rotation. Your 'small boats' and 'never frozen' angles already do the heavy lifting - they just need a system behind them.
+I can walk you through the model in 15 minutes.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Last note from me. The audit attached on Day 1 is yours to keep - the three fixes are: (1) deep-link Meta clicks to product pages, (2) concentrate Google spend on top SKU/geo clusters, (3) audit CAPI + Enhanced Conversions so Smart Bidding sees full signal.
+If the timing is wrong, no problem - the file stays accurate for roughly a quarter. If you want us to implement any of it, we can start with the tracking audit this week.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>licious-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Pure &amp; Sure</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>info@pureandsure.in</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Your Shopping clicks are being reported as organic traffic
+Day 3: The 404s that follow a theme rebuild
+Day 7: Two support addresses, one question
+Day 14: Closing the file on Pure &amp;amp; Sure</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. One finding from your live data that is worth fixing this week: your Shopping feed's tracking template writes utm_campaign=sag_organic into every paid click — I captured it on your Organic Ghee landing URL.
+In GA4 that traffic is filed as organic, so your paid Shopping investment currently looks like free traffic. The attached audit shows the exact URL and the fix.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Second finding. Five conventional paths return 404 today: /pages/contact-us, /pages/about-us, /pages/store-locator, /pages/bulk-enquiry and /pages/corporate-gifting — while /pages/contact works.
+That pattern is normal after a rebuild and invisible until a partner, a press link or a customer types the obvious URL. Redirects are an afternoon and permanent.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third note, quick. Your contact and shipping pages publish info@pureandsure.in; your cart and collection pages publish care@pureandsure.in.
+That is fine if both forward into one inbox — less fine if a customer writes to the wrong one and waits. Worth a two-minute check inside the team.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Wrapping up. Three moves: fix the sag_organic tag, redirect the five dead handles, and get a clean read on Meta so the channel question can be answered with numbers.
+If a short call on the reporting fix would be useful, I am happy to walk your team through the five-minute change.
+- Smart Pursuit, Bengaluru | 7095024220 | smartpursuit3@gmail.com</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>pure-sure-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>fresh@thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 35 live ads, 300+ cities - but the click has nowhere to land
+Day 3: The 'Find your loaf' page
+Day 7: 1M sourdoughs is a paid-media asset
+Day 14: Closing the file on The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I run paid-media audits for food brands from Bengaluru. I inspected your live footprint: 35 Google creatives under Mimansa Industries Pvt Ltd - and 1M+ sourdoughs baked, which is the strongest trust proof in Indian sourdough.
+The leak: your paid clicks do not land on a 'where is my nearest loaf' page. For a brand in 300+ cities with quick-commerce distribution, that question is the whole conversion. The buyer asks it, does not get one-tap answer, and the aggregator keeps the relationship.
+Attached is the 7-page Paid Media and Measurement Audit. Open to a short call?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+The one-page fix from the audit: a pin-code availability page that shows - in this order - nearest store, quick-commerce options, and home-delivery ETA. Pre-set the pin from the ad so the buyer lands on an answer, not a homepage.
+Everything else (creative, retargeting) amplifies this page. It is also the best email/WhatsApp capture point you have, in a weekly-repeat category.
+I can share the wireframe we would use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Quick idea from the audit. '1M+ sourdoughs baked' is stronger than any discount you can offer - it is proof. Put it in the ad hook, the landing hero, and the retargeting creative, and add a 20-second 'inside the bake' Reel at the top of the funnel.
+Bakery buyers are buying consistency and craft. You have both, and you have receipts.
+Happy to mock up three creatives around the milestone.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit stands on three fixes - (1) pin-code availability landing page for all paid traffic, (2) put the 1M+ sourdough proof into hook/hero/retargeting, (3) build the weekly repeat flow with email/WhatsApp capture.
+The audit is yours to keep. If you want us to start, the availability page is a one-week build.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>the-baker-s-dozen-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Third Wave Coffee</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>orders@thirdwavecoffee.in</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: Verified - zero live Google ads for Third Wave
+Day 3: Local campaigns for your top 10 outlets
+Day 7: Beans are a subscription, not a product
+Day 14: Closing the file on Third Wave</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I checked Google Ads Transparency for your domain this week and found zero live creatives - verified, on the Google side.
+For a brand with USD 112M raised and ~100 outlets, that means every 'coffee near me', 'cold brew delivery' and 'coffee beans online' query in your cities is answered by competitors. Local store campaigns are the cheapest walk-in channel a cafe chain can buy.
+I have attached the 7-page Paid Media and Measurement Audit, starting with the one I would run this month. To be clear about scope: this audit verifies Google - I have not claimed anything about your Meta inventory. Open to 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following the audit: the fastest win is a per-store radius campaign around your top 10 Bengaluru outlets, with a first-visit offer and measurement on store visits - not just clicks.
+Cafe chains that run local ads typically see the effect in walk-ins within the first weeks, and you can scale store by store once the template is proven.
+I can share the campaign structure and offer mechanics we would use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third idea from the audit. Your bean line competes with Blue Tokai and Sleepy Owl, who buy category search aggressively. Coffee beans are a monthly repeat purchase - the ideal profile for paid search plus a subscribe-and-save flow with free shipping.
+One more thing worth fixing before you scale spend: the storefront runs 8+ apps on an older Shopify theme. Speed multiplies every rupee of paid traffic; we would audit that first.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit's three fixes are (1) local store campaigns for the top 10 outlets, (2) a bean subscription engine with category search, (3) storefront speed before scaling spend.
+If it helps, the audit is yours to keep regardless of whether we work together. And if you want a Meta-side check as step one, we can run that in a day.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>third-wave-coffee-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Frozen Bottle</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>vipul@frozenbottle.in</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: 11 live ads for a franchise brand - the leak is in the funnel
+Day 3: The franchise funnel maths
+Day 7: Lubov deserves its own ads
+Day 14: Closing the file on Frozen Bottle</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+I audit paid media for Bengaluru food brands. I checked your live footprint: 11 Google creatives under Munchbox Frozen Foods Pvt Ltd, plus two brands (Frozen Bottle and Lubov Patisserie) and a franchise model with city and master-franchise pages.
+The gap: a single franchise sale is worth lakhs and the investor researches online first - but there is no structured paid funnel for franchise enquiries, and no store-radius campaigns for the outlets. Both are cheap to run and easy to measure.
+One small thing you can fix today: the footer links to /pages/faqs, but /pages/faq returns a 404.
+Attached is the 7-page Paid Media and Measurement Audit. Worth 15 minutes?
+- Smart Pursuit, Bengaluru | 7095024220</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following up on the audit. Compare the value of one franchise sale against the cost of a search click on 'milkshake franchise India' - the funnel pays for itself at a fraction of a single deal.
+The structure: a franchise landing page with investment range, ROI illustration and support model, Google search on franchise-intent terms, and Meta retargeting for everyone who viewed the page. Add a booking form and you have a measurable pipeline.
+Happy to share the page outline we use.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Third finding from the audit. Lubov Patisserie has its own site but no visible paid activity - it is being carried by Frozen Bottle's brand rather than having its own demand engine.
+Premium patisserie has obvious angles: occasion cakes, corporate orders and gifting. Separate creatives, separate landing pages, separate retargeting. Two brands should mean two engines.
+I can sketch the first month's creative plan if useful.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Hi team,
+Final note: the audit stands on three fixes - (1) build the franchise enquiry funnel, (2) store-radius campaigns for the top 10 outlets with per-store measurement, (3) give Lubov its own ad identity.
+The audit is yours to keep. If you want to start, the franchise funnel is the highest-value build.
+- Smart Pursuit | 7095024220</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>frozen-bottle-paid-media-measurement-audit.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>